<commit_message>
feat: update admin interface and export functionality
- Enhanced admin/index.html with improved UI
- Updated js/admin.js with expanded dashboard features
- Improved js/export.js for better data export handling
- Added and updated question data files (5S, Safety, Employee Data)
- Added Questions Full Data spreadsheet
</commit_message>
<xml_diff>
--- a/Extra Data for project/Questions files/5S اسئلة.xlsx
+++ b/Extra Data for project/Questions files/5S اسئلة.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20380"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahushu01\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Company Coding Projects\Skill Matrix Questions\skill-matrix\Extra Data for project\Questions files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BEC83E0-A955-45C4-9B39-F90F42C6312B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A77B81-61C9-4934-A2E6-4C94B652C6FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20496" windowHeight="8820" xr2:uid="{52E7F6EC-7E8A-4640-8DFE-7B3CFBB2E3A8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="1" xr2:uid="{52E7F6EC-7E8A-4640-8DFE-7B3CFBB2E3A8}"/>
   </bookViews>
   <sheets>
     <sheet name="الأسئلة" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="97">
   <si>
     <t>القسم</t>
   </si>
@@ -283,6 +284,39 @@
   </si>
   <si>
     <t>الهدف من التوحيد هو(Standardize):</t>
+  </si>
+  <si>
+    <t>Q_ID</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Opt_A</t>
+  </si>
+  <si>
+    <t>Opt_B</t>
+  </si>
+  <si>
+    <t>Opt_C</t>
+  </si>
+  <si>
+    <t>Opt_D</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>mcq</t>
+  </si>
+  <si>
+    <t>t/f</t>
   </si>
 </sst>
 </file>
@@ -765,19 +799,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D7F141D-AD7B-440E-9218-54EAB5A7B489}">
   <dimension ref="A1:I47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" style="5" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="5" customWidth="1"/>
     <col min="3" max="3" width="43" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" style="8" customWidth="1"/>
-    <col min="5" max="5" width="21.77734375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" style="8" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="14" style="8" customWidth="1"/>
-    <col min="8" max="8" width="6.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="5"/>
+    <col min="8" max="8" width="6.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -803,7 +837,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -829,7 +863,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -855,7 +889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -881,7 +915,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -907,7 +941,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -933,7 +967,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -959,7 +993,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -985,7 +1019,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
@@ -1011,7 +1045,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -1037,7 +1071,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
@@ -1063,7 +1097,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1090,7 +1124,7 @@
       </c>
       <c r="I12" s="7"/>
     </row>
-    <row r="13" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -1116,7 +1150,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -1142,7 +1176,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1168,7 +1202,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
@@ -1194,7 +1228,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
@@ -1212,7 +1246,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
@@ -1230,7 +1264,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>13</v>
       </c>
@@ -1248,7 +1282,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>13</v>
       </c>
@@ -1266,7 +1300,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
@@ -1284,7 +1318,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
@@ -1302,7 +1336,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
@@ -1320,7 +1354,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -1338,7 +1372,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>13</v>
       </c>
@@ -1356,7 +1390,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>13</v>
       </c>
@@ -1374,147 +1408,147 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="11"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="11"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="11"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="11"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="11"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
       <c r="E32" s="11"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="10"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="11"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
       <c r="E35" s="11"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
       <c r="E36" s="11"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
       <c r="E38" s="11"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
       <c r="E39" s="11"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
       <c r="D40" s="10"/>
       <c r="E40" s="11"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
       <c r="E41" s="11"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
       <c r="D42" s="10"/>
       <c r="E42" s="11"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
       <c r="D43" s="10"/>
       <c r="E43" s="11"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
       <c r="D44" s="10"/>
       <c r="E44" s="11"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
       <c r="D45" s="10"/>
       <c r="E45" s="11"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="10"/>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -1523,18 +1557,591 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="D20:G20"/>
     <mergeCell ref="D26:G26"/>
     <mergeCell ref="D21:G21"/>
     <mergeCell ref="D22:G22"/>
     <mergeCell ref="D23:G23"/>
     <mergeCell ref="D24:G24"/>
     <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="D20:G20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D27B2DE8-2C85-4A6F-BE00-AD8129579129}">
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="67.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H8" t="s">
+        <v>79</v>
+      </c>
+      <c r="I8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D10" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" t="s">
+        <v>57</v>
+      </c>
+      <c r="H11" t="s">
+        <v>58</v>
+      </c>
+      <c r="I11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H14" t="s">
+        <v>79</v>
+      </c>
+      <c r="I14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
+        <v>95</v>
+      </c>
+      <c r="D15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E15" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" t="s">
+        <v>68</v>
+      </c>
+      <c r="H15" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" t="s">
+        <v>73</v>
+      </c>
+      <c r="I16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" t="s">
+        <v>96</v>
+      </c>
+      <c r="D21" t="s">
+        <v>26</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" t="s">
+        <v>28</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" t="s">
+        <v>96</v>
+      </c>
+      <c r="D24" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" t="s">
+        <v>96</v>
+      </c>
+      <c r="D25" t="s">
+        <v>30</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" t="s">
+        <v>96</v>
+      </c>
+      <c r="D26" t="s">
+        <v>31</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>